<commit_message>
Se corrigio errores de registro de compras mediante archivos excel, ademas se agrego dos nuevas funcionalidades conbinar productos y historico de combinaciones
</commit_message>
<xml_diff>
--- a/dist/templates/plantilla_productos.xlsx
+++ b/dist/templates/plantilla_productos.xlsx
@@ -1,203 +1,194 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\CarePharm\dist\templates\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3316A7C-942F-439E-BB8C-0B51C7E05B43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LISTA EXCEL" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
-  <si>
-    <t xml:space="preserve">COD.DIGEMID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRODUCTO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DESCRIPCION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRESENTACION/FORMAS POR UNIDAD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LABORATORIO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F.V.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CANT x CAJA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CANT. UNI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LOT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PREC.PROVEEDOR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRECIO UNITARIO (PRECIO COSTO)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FACTURA Nro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nro DE GUIA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRECIO VTA.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRECIO VTA. COMERCIAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CODIGO DE BARRAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PROVEEDOR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RUC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEDE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F.COMPRA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REGISTRO SA.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cod_digemid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">presentation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">laboratorio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fecha_venc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cant_caja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stock</t>
-  </si>
-  <si>
-    <t xml:space="preserve">num_lote</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prec_prov</t>
-  </si>
-  <si>
-    <t xml:space="preserve">price_in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nro_factura</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nro_guia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">price_out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">price_may</t>
-  </si>
-  <si>
-    <t xml:space="preserve">barcode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">proveedor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ruc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sede</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fecha_compra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">reg_san</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1211041</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BICARBONATO DE SODIO POTE X 500</t>
-  </si>
-  <si>
-    <t xml:space="preserve">POTE X 50 GR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OLCASA S.A.C.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1/25/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">35167</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S/ 15.96</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S/ 1.13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F001-0000857</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S/ 2.00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S/ 1.80</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.9641-15 F001-0000657</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2300657+90</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IQUITOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5/05/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">123456</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+  <si>
+    <t>COD.DIGEMID</t>
+  </si>
+  <si>
+    <t>PRODUCTO</t>
+  </si>
+  <si>
+    <t>DESCRIPCION</t>
+  </si>
+  <si>
+    <t>PRESENTACION/FORMAS POR UNIDAD</t>
+  </si>
+  <si>
+    <t>LABORATORIO</t>
+  </si>
+  <si>
+    <t>F.V.</t>
+  </si>
+  <si>
+    <t>CANT x CAJA</t>
+  </si>
+  <si>
+    <t>CANT. UNI</t>
+  </si>
+  <si>
+    <t>LOT</t>
+  </si>
+  <si>
+    <t>PREC.PROVEEDOR</t>
+  </si>
+  <si>
+    <t>PRECIO UNITARIO (PRECIO COSTO)</t>
+  </si>
+  <si>
+    <t>FACTURA Nro</t>
+  </si>
+  <si>
+    <t>Nro DE GUIA</t>
+  </si>
+  <si>
+    <t>PRECIO VTA.</t>
+  </si>
+  <si>
+    <t>PRECIO VTA. COMERCIAL</t>
+  </si>
+  <si>
+    <t>CODIGO DE BARRAS</t>
+  </si>
+  <si>
+    <t>PROVEEDOR</t>
+  </si>
+  <si>
+    <t>RUC</t>
+  </si>
+  <si>
+    <t>SEDE</t>
+  </si>
+  <si>
+    <t>F.COMPRA</t>
+  </si>
+  <si>
+    <t>REGISTRO SA.</t>
+  </si>
+  <si>
+    <t>cod_digemid</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>presentation</t>
+  </si>
+  <si>
+    <t>laboratorio</t>
+  </si>
+  <si>
+    <t>fecha_venc</t>
+  </si>
+  <si>
+    <t>cant_caja</t>
+  </si>
+  <si>
+    <t>stock</t>
+  </si>
+  <si>
+    <t>num_lote</t>
+  </si>
+  <si>
+    <t>prec_prov</t>
+  </si>
+  <si>
+    <t>price_in</t>
+  </si>
+  <si>
+    <t>nro_factura</t>
+  </si>
+  <si>
+    <t>nro_guia</t>
+  </si>
+  <si>
+    <t>price_out</t>
+  </si>
+  <si>
+    <t>price_may</t>
+  </si>
+  <si>
+    <t>barcode</t>
+  </si>
+  <si>
+    <t>proveedor</t>
+  </si>
+  <si>
+    <t>ruc</t>
+  </si>
+  <si>
+    <t>sede</t>
+  </si>
+  <si>
+    <t>fecha_compra</t>
+  </si>
+  <si>
+    <t>reg_san</t>
+  </si>
+  <si>
+    <t>OLCASA S.A.C.</t>
+  </si>
+  <si>
+    <t>1/25/2026</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>35167</t>
+  </si>
+  <si>
+    <t>F001-0000857</t>
+  </si>
+  <si>
+    <t>IQUITOS</t>
+  </si>
+  <si>
+    <t>5/05/2026</t>
+  </si>
+  <si>
+    <t>BICARBONATO DE SODIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> POTE X 50G</t>
+  </si>
+  <si>
+    <t>E-12345</t>
+  </si>
+  <si>
+    <t>ROXFARMA S.A</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="8" formatCode="&quot;S/&quot;\ #,##0.00;[Red]\-&quot;S/&quot;\ #,##0.00"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="9"/>
       <name val="Calibri"/>
@@ -207,16 +198,19 @@
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
+      <i/>
       <sz val="8"/>
       <color rgb="FF666666"/>
       <name val="Calibri"/>
-      <i/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="11">
@@ -299,7 +293,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -328,229 +322,536 @@
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="8" fontId="3" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="44546A"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E7E6E6"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4472C4"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="ED7D31"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A5A5A5"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="FFC000"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="5B9BD5"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="70AD47"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0563C1"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="954F72"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:U103"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="26" customWidth="1"/>
-    <col min="12" max="12" width="18" customWidth="1"/>
-    <col min="13" max="13" width="16" customWidth="1"/>
-    <col min="14" max="14" width="14" customWidth="1"/>
-    <col min="15" max="15" width="22" customWidth="1"/>
-    <col min="16" max="16" width="20" customWidth="1"/>
-    <col min="17" max="17" width="28" customWidth="1"/>
-    <col min="18" max="18" width="16" customWidth="1"/>
-    <col min="19" max="19" width="14" customWidth="1"/>
-    <col min="20" max="20" width="14" customWidth="1"/>
-    <col min="21" max="21" width="18" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="8" width="14" customWidth="1"/>
+    <col min="9" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="26" customWidth="1"/>
+    <col min="13" max="13" width="18" customWidth="1"/>
+    <col min="14" max="14" width="16" customWidth="1"/>
+    <col min="15" max="15" width="14" customWidth="1"/>
+    <col min="16" max="16" width="22" customWidth="1"/>
+    <col min="17" max="17" width="20" customWidth="1"/>
+    <col min="18" max="18" width="28" customWidth="1"/>
+    <col min="19" max="19" width="16" customWidth="1"/>
+    <col min="20" max="21" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="42" customHeight="1">
-      <c r="A1" t="s" s="1">
+    <row r="1" spans="1:21" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="1">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="1">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s" s="1">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s" s="2">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s" s="3">
+      <c r="F1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s" s="4">
+      <c r="H1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s" s="4">
+      <c r="I1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s" s="4">
+      <c r="J1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s" s="4">
+      <c r="K1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s" s="5">
+      <c r="L1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s" s="2">
+      <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s" s="2">
+      <c r="N1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s" s="6">
+      <c r="O1" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s" s="6">
+      <c r="P1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s" s="1">
+      <c r="Q1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s" s="2">
+      <c r="R1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s" s="2">
+      <c r="S1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s" s="4">
+      <c r="T1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s" s="3">
+      <c r="U1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" ht="13">
-      <c r="A2" t="s" s="7">
+    </row>
+    <row r="2" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B2" t="s" s="7">
+      <c r="B2" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C2" t="s" s="7">
+      <c r="C2" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D2" t="s" s="7">
+      <c r="D2" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E2" t="s" s="7">
+      <c r="E2" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="F2" t="s" s="7">
+      <c r="F2" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G2" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="G2" t="s" s="7">
+      <c r="H2" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="H2" t="s" s="7">
+      <c r="I2" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="I2" t="s" s="7">
+      <c r="J2" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="J2" t="s" s="7">
+      <c r="K2" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="K2" t="s" s="7">
+      <c r="L2" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="L2" t="s" s="7">
+      <c r="M2" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="M2" t="s" s="7">
+      <c r="N2" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="N2" t="s" s="7">
+      <c r="O2" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="O2" t="s" s="7">
+      <c r="P2" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="P2" t="s" s="7">
+      <c r="Q2" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="Q2" t="s" s="7">
+      <c r="R2" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="R2" t="s" s="7">
+      <c r="S2" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="S2" t="s" s="7">
+      <c r="T2" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="T2" t="s" s="7">
+      <c r="U2" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="U2" t="s" s="7">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="3" ht="16">
-      <c r="A3" t="s" s="8">
+    </row>
+    <row r="3" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B3" t="s" s="8">
+      <c r="F3" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="G3" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="C3" t="s" s="8">
-        <v>43</v>
-      </c>
-      <c r="D3" t="s" s="8">
+      <c r="H3" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="E3" t="s" s="8">
+      <c r="I3" s="8">
+        <v>10</v>
+      </c>
+      <c r="J3" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="F3" t="s" s="8">
+      <c r="K3" s="10">
+        <v>13.56</v>
+      </c>
+      <c r="L3" s="8">
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="M3" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="G3" t="s" s="8">
+      <c r="N3" s="9"/>
+      <c r="O3" s="8">
+        <v>3</v>
+      </c>
+      <c r="P3" s="8">
+        <v>2.8</v>
+      </c>
+      <c r="Q3" s="8">
+        <v>77021159626955</v>
+      </c>
+      <c r="R3" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="S3" s="9">
+        <v>20101348203</v>
+      </c>
+      <c r="T3" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="H3" t="s" s="8">
+      <c r="U3" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="I3" t="s" s="8">
-        <v>49</v>
-      </c>
-      <c r="J3" t="s" s="8">
-        <v>50</v>
-      </c>
-      <c r="K3" t="s" s="8">
-        <v>51</v>
-      </c>
-      <c r="L3" t="s" s="8">
-        <v>52</v>
-      </c>
-      <c r="M3" s="9"/>
-      <c r="N3" t="s" s="8">
-        <v>53</v>
-      </c>
-      <c r="O3" t="s" s="8">
-        <v>54</v>
-      </c>
-      <c r="P3" t="s" s="8">
-        <v>55</v>
-      </c>
-      <c r="Q3" t="s" s="8">
-        <v>56</v>
-      </c>
-      <c r="R3" s="9"/>
-      <c r="S3" t="s" s="8">
-        <v>57</v>
-      </c>
-      <c r="T3" t="s" s="8">
-        <v>58</v>
-      </c>
-      <c r="U3" t="s" s="8">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="4" ht="15">
+    </row>
+    <row r="4" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A4" s="9"/>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
@@ -573,7 +874,7 @@
       <c r="T4" s="9"/>
       <c r="U4" s="9"/>
     </row>
-    <row r="5" ht="15">
+    <row r="5" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A5" s="9"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
@@ -596,7 +897,7 @@
       <c r="T5" s="9"/>
       <c r="U5" s="9"/>
     </row>
-    <row r="6" ht="15">
+    <row r="6" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A6" s="9"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -619,7 +920,7 @@
       <c r="T6" s="9"/>
       <c r="U6" s="9"/>
     </row>
-    <row r="7" ht="15">
+    <row r="7" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A7" s="9"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
@@ -642,7 +943,7 @@
       <c r="T7" s="9"/>
       <c r="U7" s="9"/>
     </row>
-    <row r="8" ht="15">
+    <row r="8" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A8" s="9"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -665,7 +966,7 @@
       <c r="T8" s="9"/>
       <c r="U8" s="9"/>
     </row>
-    <row r="9" ht="15">
+    <row r="9" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A9" s="9"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -688,7 +989,7 @@
       <c r="T9" s="9"/>
       <c r="U9" s="9"/>
     </row>
-    <row r="10" ht="15">
+    <row r="10" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A10" s="9"/>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -711,7 +1012,7 @@
       <c r="T10" s="9"/>
       <c r="U10" s="9"/>
     </row>
-    <row r="11" ht="15">
+    <row r="11" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A11" s="9"/>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
@@ -734,7 +1035,7 @@
       <c r="T11" s="9"/>
       <c r="U11" s="9"/>
     </row>
-    <row r="12" ht="15">
+    <row r="12" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A12" s="9"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -757,7 +1058,7 @@
       <c r="T12" s="9"/>
       <c r="U12" s="9"/>
     </row>
-    <row r="13" ht="15">
+    <row r="13" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A13" s="9"/>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -780,7 +1081,7 @@
       <c r="T13" s="9"/>
       <c r="U13" s="9"/>
     </row>
-    <row r="14" ht="15">
+    <row r="14" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A14" s="9"/>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -803,7 +1104,7 @@
       <c r="T14" s="9"/>
       <c r="U14" s="9"/>
     </row>
-    <row r="15" ht="15">
+    <row r="15" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A15" s="9"/>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -826,7 +1127,7 @@
       <c r="T15" s="9"/>
       <c r="U15" s="9"/>
     </row>
-    <row r="16" ht="15">
+    <row r="16" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A16" s="9"/>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -849,7 +1150,7 @@
       <c r="T16" s="9"/>
       <c r="U16" s="9"/>
     </row>
-    <row r="17" ht="15">
+    <row r="17" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A17" s="9"/>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
@@ -872,7 +1173,7 @@
       <c r="T17" s="9"/>
       <c r="U17" s="9"/>
     </row>
-    <row r="18" ht="15">
+    <row r="18" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A18" s="9"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -895,7 +1196,7 @@
       <c r="T18" s="9"/>
       <c r="U18" s="9"/>
     </row>
-    <row r="19" ht="15">
+    <row r="19" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A19" s="9"/>
       <c r="B19" s="9"/>
       <c r="C19" s="9"/>
@@ -918,7 +1219,7 @@
       <c r="T19" s="9"/>
       <c r="U19" s="9"/>
     </row>
-    <row r="20" ht="15">
+    <row r="20" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A20" s="9"/>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
@@ -941,7 +1242,7 @@
       <c r="T20" s="9"/>
       <c r="U20" s="9"/>
     </row>
-    <row r="21" ht="15">
+    <row r="21" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A21" s="9"/>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
@@ -964,7 +1265,7 @@
       <c r="T21" s="9"/>
       <c r="U21" s="9"/>
     </row>
-    <row r="22" ht="15">
+    <row r="22" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A22" s="9"/>
       <c r="B22" s="9"/>
       <c r="C22" s="9"/>
@@ -987,7 +1288,7 @@
       <c r="T22" s="9"/>
       <c r="U22" s="9"/>
     </row>
-    <row r="23" ht="15">
+    <row r="23" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A23" s="9"/>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
@@ -1010,7 +1311,7 @@
       <c r="T23" s="9"/>
       <c r="U23" s="9"/>
     </row>
-    <row r="24" ht="15">
+    <row r="24" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A24" s="9"/>
       <c r="B24" s="9"/>
       <c r="C24" s="9"/>
@@ -1033,7 +1334,7 @@
       <c r="T24" s="9"/>
       <c r="U24" s="9"/>
     </row>
-    <row r="25" ht="15">
+    <row r="25" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A25" s="9"/>
       <c r="B25" s="9"/>
       <c r="C25" s="9"/>
@@ -1056,7 +1357,7 @@
       <c r="T25" s="9"/>
       <c r="U25" s="9"/>
     </row>
-    <row r="26" ht="15">
+    <row r="26" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A26" s="9"/>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
@@ -1079,7 +1380,7 @@
       <c r="T26" s="9"/>
       <c r="U26" s="9"/>
     </row>
-    <row r="27" ht="15">
+    <row r="27" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A27" s="9"/>
       <c r="B27" s="9"/>
       <c r="C27" s="9"/>
@@ -1102,7 +1403,7 @@
       <c r="T27" s="9"/>
       <c r="U27" s="9"/>
     </row>
-    <row r="28" ht="15">
+    <row r="28" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A28" s="9"/>
       <c r="B28" s="9"/>
       <c r="C28" s="9"/>
@@ -1125,7 +1426,7 @@
       <c r="T28" s="9"/>
       <c r="U28" s="9"/>
     </row>
-    <row r="29" ht="15">
+    <row r="29" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A29" s="9"/>
       <c r="B29" s="9"/>
       <c r="C29" s="9"/>
@@ -1148,7 +1449,7 @@
       <c r="T29" s="9"/>
       <c r="U29" s="9"/>
     </row>
-    <row r="30" ht="15">
+    <row r="30" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A30" s="9"/>
       <c r="B30" s="9"/>
       <c r="C30" s="9"/>
@@ -1171,7 +1472,7 @@
       <c r="T30" s="9"/>
       <c r="U30" s="9"/>
     </row>
-    <row r="31" ht="15">
+    <row r="31" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A31" s="9"/>
       <c r="B31" s="9"/>
       <c r="C31" s="9"/>
@@ -1194,7 +1495,7 @@
       <c r="T31" s="9"/>
       <c r="U31" s="9"/>
     </row>
-    <row r="32" ht="15">
+    <row r="32" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A32" s="9"/>
       <c r="B32" s="9"/>
       <c r="C32" s="9"/>
@@ -1217,7 +1518,7 @@
       <c r="T32" s="9"/>
       <c r="U32" s="9"/>
     </row>
-    <row r="33" ht="15">
+    <row r="33" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A33" s="9"/>
       <c r="B33" s="9"/>
       <c r="C33" s="9"/>
@@ -1240,7 +1541,7 @@
       <c r="T33" s="9"/>
       <c r="U33" s="9"/>
     </row>
-    <row r="34" ht="15">
+    <row r="34" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A34" s="9"/>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -1263,7 +1564,7 @@
       <c r="T34" s="9"/>
       <c r="U34" s="9"/>
     </row>
-    <row r="35" ht="15">
+    <row r="35" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A35" s="9"/>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
@@ -1286,7 +1587,7 @@
       <c r="T35" s="9"/>
       <c r="U35" s="9"/>
     </row>
-    <row r="36" ht="15">
+    <row r="36" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A36" s="9"/>
       <c r="B36" s="9"/>
       <c r="C36" s="9"/>
@@ -1309,7 +1610,7 @@
       <c r="T36" s="9"/>
       <c r="U36" s="9"/>
     </row>
-    <row r="37" ht="15">
+    <row r="37" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A37" s="9"/>
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
@@ -1332,7 +1633,7 @@
       <c r="T37" s="9"/>
       <c r="U37" s="9"/>
     </row>
-    <row r="38" ht="15">
+    <row r="38" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A38" s="9"/>
       <c r="B38" s="9"/>
       <c r="C38" s="9"/>
@@ -1355,7 +1656,7 @@
       <c r="T38" s="9"/>
       <c r="U38" s="9"/>
     </row>
-    <row r="39" ht="15">
+    <row r="39" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A39" s="9"/>
       <c r="B39" s="9"/>
       <c r="C39" s="9"/>
@@ -1378,7 +1679,7 @@
       <c r="T39" s="9"/>
       <c r="U39" s="9"/>
     </row>
-    <row r="40" ht="15">
+    <row r="40" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A40" s="9"/>
       <c r="B40" s="9"/>
       <c r="C40" s="9"/>
@@ -1401,7 +1702,7 @@
       <c r="T40" s="9"/>
       <c r="U40" s="9"/>
     </row>
-    <row r="41" ht="15">
+    <row r="41" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A41" s="9"/>
       <c r="B41" s="9"/>
       <c r="C41" s="9"/>
@@ -1424,7 +1725,7 @@
       <c r="T41" s="9"/>
       <c r="U41" s="9"/>
     </row>
-    <row r="42" ht="15">
+    <row r="42" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A42" s="9"/>
       <c r="B42" s="9"/>
       <c r="C42" s="9"/>
@@ -1447,7 +1748,7 @@
       <c r="T42" s="9"/>
       <c r="U42" s="9"/>
     </row>
-    <row r="43" ht="15">
+    <row r="43" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A43" s="9"/>
       <c r="B43" s="9"/>
       <c r="C43" s="9"/>
@@ -1470,7 +1771,7 @@
       <c r="T43" s="9"/>
       <c r="U43" s="9"/>
     </row>
-    <row r="44" ht="15">
+    <row r="44" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A44" s="9"/>
       <c r="B44" s="9"/>
       <c r="C44" s="9"/>
@@ -1493,7 +1794,7 @@
       <c r="T44" s="9"/>
       <c r="U44" s="9"/>
     </row>
-    <row r="45" ht="15">
+    <row r="45" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A45" s="9"/>
       <c r="B45" s="9"/>
       <c r="C45" s="9"/>
@@ -1516,7 +1817,7 @@
       <c r="T45" s="9"/>
       <c r="U45" s="9"/>
     </row>
-    <row r="46" ht="15">
+    <row r="46" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A46" s="9"/>
       <c r="B46" s="9"/>
       <c r="C46" s="9"/>
@@ -1539,7 +1840,7 @@
       <c r="T46" s="9"/>
       <c r="U46" s="9"/>
     </row>
-    <row r="47" ht="15">
+    <row r="47" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A47" s="9"/>
       <c r="B47" s="9"/>
       <c r="C47" s="9"/>
@@ -1562,7 +1863,7 @@
       <c r="T47" s="9"/>
       <c r="U47" s="9"/>
     </row>
-    <row r="48" ht="15">
+    <row r="48" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A48" s="9"/>
       <c r="B48" s="9"/>
       <c r="C48" s="9"/>
@@ -1585,7 +1886,7 @@
       <c r="T48" s="9"/>
       <c r="U48" s="9"/>
     </row>
-    <row r="49" ht="15">
+    <row r="49" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A49" s="9"/>
       <c r="B49" s="9"/>
       <c r="C49" s="9"/>
@@ -1608,7 +1909,7 @@
       <c r="T49" s="9"/>
       <c r="U49" s="9"/>
     </row>
-    <row r="50" ht="15">
+    <row r="50" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A50" s="9"/>
       <c r="B50" s="9"/>
       <c r="C50" s="9"/>
@@ -1631,7 +1932,7 @@
       <c r="T50" s="9"/>
       <c r="U50" s="9"/>
     </row>
-    <row r="51" ht="15">
+    <row r="51" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A51" s="9"/>
       <c r="B51" s="9"/>
       <c r="C51" s="9"/>
@@ -1654,7 +1955,7 @@
       <c r="T51" s="9"/>
       <c r="U51" s="9"/>
     </row>
-    <row r="52" ht="15">
+    <row r="52" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A52" s="9"/>
       <c r="B52" s="9"/>
       <c r="C52" s="9"/>
@@ -1677,7 +1978,7 @@
       <c r="T52" s="9"/>
       <c r="U52" s="9"/>
     </row>
-    <row r="53" ht="15">
+    <row r="53" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A53" s="9"/>
       <c r="B53" s="9"/>
       <c r="C53" s="9"/>
@@ -1700,7 +2001,7 @@
       <c r="T53" s="9"/>
       <c r="U53" s="9"/>
     </row>
-    <row r="54" ht="15">
+    <row r="54" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A54" s="9"/>
       <c r="B54" s="9"/>
       <c r="C54" s="9"/>
@@ -1723,7 +2024,7 @@
       <c r="T54" s="9"/>
       <c r="U54" s="9"/>
     </row>
-    <row r="55" ht="15">
+    <row r="55" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A55" s="9"/>
       <c r="B55" s="9"/>
       <c r="C55" s="9"/>
@@ -1746,7 +2047,7 @@
       <c r="T55" s="9"/>
       <c r="U55" s="9"/>
     </row>
-    <row r="56" ht="15">
+    <row r="56" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A56" s="9"/>
       <c r="B56" s="9"/>
       <c r="C56" s="9"/>
@@ -1769,7 +2070,7 @@
       <c r="T56" s="9"/>
       <c r="U56" s="9"/>
     </row>
-    <row r="57" ht="15">
+    <row r="57" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A57" s="9"/>
       <c r="B57" s="9"/>
       <c r="C57" s="9"/>
@@ -1792,7 +2093,7 @@
       <c r="T57" s="9"/>
       <c r="U57" s="9"/>
     </row>
-    <row r="58" ht="15">
+    <row r="58" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A58" s="9"/>
       <c r="B58" s="9"/>
       <c r="C58" s="9"/>
@@ -1815,7 +2116,7 @@
       <c r="T58" s="9"/>
       <c r="U58" s="9"/>
     </row>
-    <row r="59" ht="15">
+    <row r="59" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A59" s="9"/>
       <c r="B59" s="9"/>
       <c r="C59" s="9"/>
@@ -1838,7 +2139,7 @@
       <c r="T59" s="9"/>
       <c r="U59" s="9"/>
     </row>
-    <row r="60" ht="15">
+    <row r="60" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A60" s="9"/>
       <c r="B60" s="9"/>
       <c r="C60" s="9"/>
@@ -1861,7 +2162,7 @@
       <c r="T60" s="9"/>
       <c r="U60" s="9"/>
     </row>
-    <row r="61" ht="15">
+    <row r="61" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A61" s="9"/>
       <c r="B61" s="9"/>
       <c r="C61" s="9"/>
@@ -1884,7 +2185,7 @@
       <c r="T61" s="9"/>
       <c r="U61" s="9"/>
     </row>
-    <row r="62" ht="15">
+    <row r="62" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A62" s="9"/>
       <c r="B62" s="9"/>
       <c r="C62" s="9"/>
@@ -1907,7 +2208,7 @@
       <c r="T62" s="9"/>
       <c r="U62" s="9"/>
     </row>
-    <row r="63" ht="15">
+    <row r="63" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A63" s="9"/>
       <c r="B63" s="9"/>
       <c r="C63" s="9"/>
@@ -1930,7 +2231,7 @@
       <c r="T63" s="9"/>
       <c r="U63" s="9"/>
     </row>
-    <row r="64" ht="15">
+    <row r="64" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A64" s="9"/>
       <c r="B64" s="9"/>
       <c r="C64" s="9"/>
@@ -1953,7 +2254,7 @@
       <c r="T64" s="9"/>
       <c r="U64" s="9"/>
     </row>
-    <row r="65" ht="15">
+    <row r="65" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A65" s="9"/>
       <c r="B65" s="9"/>
       <c r="C65" s="9"/>
@@ -1976,7 +2277,7 @@
       <c r="T65" s="9"/>
       <c r="U65" s="9"/>
     </row>
-    <row r="66" ht="15">
+    <row r="66" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A66" s="9"/>
       <c r="B66" s="9"/>
       <c r="C66" s="9"/>
@@ -1999,7 +2300,7 @@
       <c r="T66" s="9"/>
       <c r="U66" s="9"/>
     </row>
-    <row r="67" ht="15">
+    <row r="67" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A67" s="9"/>
       <c r="B67" s="9"/>
       <c r="C67" s="9"/>
@@ -2022,7 +2323,7 @@
       <c r="T67" s="9"/>
       <c r="U67" s="9"/>
     </row>
-    <row r="68" ht="15">
+    <row r="68" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A68" s="9"/>
       <c r="B68" s="9"/>
       <c r="C68" s="9"/>
@@ -2045,7 +2346,7 @@
       <c r="T68" s="9"/>
       <c r="U68" s="9"/>
     </row>
-    <row r="69" ht="15">
+    <row r="69" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A69" s="9"/>
       <c r="B69" s="9"/>
       <c r="C69" s="9"/>
@@ -2068,7 +2369,7 @@
       <c r="T69" s="9"/>
       <c r="U69" s="9"/>
     </row>
-    <row r="70" ht="15">
+    <row r="70" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A70" s="9"/>
       <c r="B70" s="9"/>
       <c r="C70" s="9"/>
@@ -2091,7 +2392,7 @@
       <c r="T70" s="9"/>
       <c r="U70" s="9"/>
     </row>
-    <row r="71" ht="15">
+    <row r="71" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A71" s="9"/>
       <c r="B71" s="9"/>
       <c r="C71" s="9"/>
@@ -2114,7 +2415,7 @@
       <c r="T71" s="9"/>
       <c r="U71" s="9"/>
     </row>
-    <row r="72" ht="15">
+    <row r="72" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A72" s="9"/>
       <c r="B72" s="9"/>
       <c r="C72" s="9"/>
@@ -2137,7 +2438,7 @@
       <c r="T72" s="9"/>
       <c r="U72" s="9"/>
     </row>
-    <row r="73" ht="15">
+    <row r="73" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A73" s="9"/>
       <c r="B73" s="9"/>
       <c r="C73" s="9"/>
@@ -2160,7 +2461,7 @@
       <c r="T73" s="9"/>
       <c r="U73" s="9"/>
     </row>
-    <row r="74" ht="15">
+    <row r="74" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A74" s="9"/>
       <c r="B74" s="9"/>
       <c r="C74" s="9"/>
@@ -2183,7 +2484,7 @@
       <c r="T74" s="9"/>
       <c r="U74" s="9"/>
     </row>
-    <row r="75" ht="15">
+    <row r="75" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A75" s="9"/>
       <c r="B75" s="9"/>
       <c r="C75" s="9"/>
@@ -2206,7 +2507,7 @@
       <c r="T75" s="9"/>
       <c r="U75" s="9"/>
     </row>
-    <row r="76" ht="15">
+    <row r="76" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A76" s="9"/>
       <c r="B76" s="9"/>
       <c r="C76" s="9"/>
@@ -2229,7 +2530,7 @@
       <c r="T76" s="9"/>
       <c r="U76" s="9"/>
     </row>
-    <row r="77" ht="15">
+    <row r="77" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A77" s="9"/>
       <c r="B77" s="9"/>
       <c r="C77" s="9"/>
@@ -2252,7 +2553,7 @@
       <c r="T77" s="9"/>
       <c r="U77" s="9"/>
     </row>
-    <row r="78" ht="15">
+    <row r="78" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A78" s="9"/>
       <c r="B78" s="9"/>
       <c r="C78" s="9"/>
@@ -2275,7 +2576,7 @@
       <c r="T78" s="9"/>
       <c r="U78" s="9"/>
     </row>
-    <row r="79" ht="15">
+    <row r="79" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A79" s="9"/>
       <c r="B79" s="9"/>
       <c r="C79" s="9"/>
@@ -2298,7 +2599,7 @@
       <c r="T79" s="9"/>
       <c r="U79" s="9"/>
     </row>
-    <row r="80" ht="15">
+    <row r="80" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A80" s="9"/>
       <c r="B80" s="9"/>
       <c r="C80" s="9"/>
@@ -2321,7 +2622,7 @@
       <c r="T80" s="9"/>
       <c r="U80" s="9"/>
     </row>
-    <row r="81" ht="15">
+    <row r="81" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A81" s="9"/>
       <c r="B81" s="9"/>
       <c r="C81" s="9"/>
@@ -2344,7 +2645,7 @@
       <c r="T81" s="9"/>
       <c r="U81" s="9"/>
     </row>
-    <row r="82" ht="15">
+    <row r="82" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A82" s="9"/>
       <c r="B82" s="9"/>
       <c r="C82" s="9"/>
@@ -2367,7 +2668,7 @@
       <c r="T82" s="9"/>
       <c r="U82" s="9"/>
     </row>
-    <row r="83" ht="15">
+    <row r="83" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A83" s="9"/>
       <c r="B83" s="9"/>
       <c r="C83" s="9"/>
@@ -2390,7 +2691,7 @@
       <c r="T83" s="9"/>
       <c r="U83" s="9"/>
     </row>
-    <row r="84" ht="15">
+    <row r="84" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A84" s="9"/>
       <c r="B84" s="9"/>
       <c r="C84" s="9"/>
@@ -2413,7 +2714,7 @@
       <c r="T84" s="9"/>
       <c r="U84" s="9"/>
     </row>
-    <row r="85" ht="15">
+    <row r="85" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A85" s="9"/>
       <c r="B85" s="9"/>
       <c r="C85" s="9"/>
@@ -2436,7 +2737,7 @@
       <c r="T85" s="9"/>
       <c r="U85" s="9"/>
     </row>
-    <row r="86" ht="15">
+    <row r="86" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A86" s="9"/>
       <c r="B86" s="9"/>
       <c r="C86" s="9"/>
@@ -2459,7 +2760,7 @@
       <c r="T86" s="9"/>
       <c r="U86" s="9"/>
     </row>
-    <row r="87" ht="15">
+    <row r="87" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A87" s="9"/>
       <c r="B87" s="9"/>
       <c r="C87" s="9"/>
@@ -2482,7 +2783,7 @@
       <c r="T87" s="9"/>
       <c r="U87" s="9"/>
     </row>
-    <row r="88" ht="15">
+    <row r="88" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A88" s="9"/>
       <c r="B88" s="9"/>
       <c r="C88" s="9"/>
@@ -2505,7 +2806,7 @@
       <c r="T88" s="9"/>
       <c r="U88" s="9"/>
     </row>
-    <row r="89" ht="15">
+    <row r="89" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A89" s="9"/>
       <c r="B89" s="9"/>
       <c r="C89" s="9"/>
@@ -2528,7 +2829,7 @@
       <c r="T89" s="9"/>
       <c r="U89" s="9"/>
     </row>
-    <row r="90" ht="15">
+    <row r="90" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A90" s="9"/>
       <c r="B90" s="9"/>
       <c r="C90" s="9"/>
@@ -2551,7 +2852,7 @@
       <c r="T90" s="9"/>
       <c r="U90" s="9"/>
     </row>
-    <row r="91" ht="15">
+    <row r="91" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A91" s="9"/>
       <c r="B91" s="9"/>
       <c r="C91" s="9"/>
@@ -2574,7 +2875,7 @@
       <c r="T91" s="9"/>
       <c r="U91" s="9"/>
     </row>
-    <row r="92" ht="15">
+    <row r="92" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A92" s="9"/>
       <c r="B92" s="9"/>
       <c r="C92" s="9"/>
@@ -2597,7 +2898,7 @@
       <c r="T92" s="9"/>
       <c r="U92" s="9"/>
     </row>
-    <row r="93" ht="15">
+    <row r="93" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A93" s="9"/>
       <c r="B93" s="9"/>
       <c r="C93" s="9"/>
@@ -2620,7 +2921,7 @@
       <c r="T93" s="9"/>
       <c r="U93" s="9"/>
     </row>
-    <row r="94" ht="15">
+    <row r="94" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A94" s="9"/>
       <c r="B94" s="9"/>
       <c r="C94" s="9"/>
@@ -2643,7 +2944,7 @@
       <c r="T94" s="9"/>
       <c r="U94" s="9"/>
     </row>
-    <row r="95" ht="15">
+    <row r="95" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A95" s="9"/>
       <c r="B95" s="9"/>
       <c r="C95" s="9"/>
@@ -2666,7 +2967,7 @@
       <c r="T95" s="9"/>
       <c r="U95" s="9"/>
     </row>
-    <row r="96" ht="15">
+    <row r="96" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A96" s="9"/>
       <c r="B96" s="9"/>
       <c r="C96" s="9"/>
@@ -2689,7 +2990,7 @@
       <c r="T96" s="9"/>
       <c r="U96" s="9"/>
     </row>
-    <row r="97" ht="15">
+    <row r="97" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A97" s="9"/>
       <c r="B97" s="9"/>
       <c r="C97" s="9"/>
@@ -2712,7 +3013,7 @@
       <c r="T97" s="9"/>
       <c r="U97" s="9"/>
     </row>
-    <row r="98" ht="15">
+    <row r="98" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A98" s="9"/>
       <c r="B98" s="9"/>
       <c r="C98" s="9"/>
@@ -2735,7 +3036,7 @@
       <c r="T98" s="9"/>
       <c r="U98" s="9"/>
     </row>
-    <row r="99" ht="15">
+    <row r="99" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A99" s="9"/>
       <c r="B99" s="9"/>
       <c r="C99" s="9"/>
@@ -2758,7 +3059,7 @@
       <c r="T99" s="9"/>
       <c r="U99" s="9"/>
     </row>
-    <row r="100" ht="15">
+    <row r="100" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A100" s="9"/>
       <c r="B100" s="9"/>
       <c r="C100" s="9"/>
@@ -2781,7 +3082,7 @@
       <c r="T100" s="9"/>
       <c r="U100" s="9"/>
     </row>
-    <row r="101" ht="15">
+    <row r="101" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A101" s="9"/>
       <c r="B101" s="9"/>
       <c r="C101" s="9"/>
@@ -2804,7 +3105,7 @@
       <c r="T101" s="9"/>
       <c r="U101" s="9"/>
     </row>
-    <row r="102" ht="15">
+    <row r="102" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A102" s="9"/>
       <c r="B102" s="9"/>
       <c r="C102" s="9"/>
@@ -2827,7 +3128,7 @@
       <c r="T102" s="9"/>
       <c r="U102" s="9"/>
     </row>
-    <row r="103" ht="15">
+    <row r="103" spans="1:21" ht="12" x14ac:dyDescent="0.2">
       <c r="A103" s="9"/>
       <c r="B103" s="9"/>
       <c r="C103" s="9"/>
@@ -2851,6 +3152,7 @@
       <c r="U103" s="9"/>
     </row>
   </sheetData>
-  <pageSetup orientation="landscape" paperSize="9"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Se quito columna descripcion y se agrego en su lugar principio activo
</commit_message>
<xml_diff>
--- a/dist/templates/plantilla_productos.xlsx
+++ b/dist/templates/plantilla_productos.xlsx
@@ -1,194 +1,206 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\CarePharm\dist\templates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3316A7C-942F-439E-BB8C-0B51C7E05B43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LISTA EXCEL" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
-  <si>
-    <t>COD.DIGEMID</t>
-  </si>
-  <si>
-    <t>PRODUCTO</t>
-  </si>
-  <si>
-    <t>DESCRIPCION</t>
-  </si>
-  <si>
-    <t>PRESENTACION/FORMAS POR UNIDAD</t>
-  </si>
-  <si>
-    <t>LABORATORIO</t>
-  </si>
-  <si>
-    <t>F.V.</t>
-  </si>
-  <si>
-    <t>CANT x CAJA</t>
-  </si>
-  <si>
-    <t>CANT. UNI</t>
-  </si>
-  <si>
-    <t>LOT</t>
-  </si>
-  <si>
-    <t>PREC.PROVEEDOR</t>
-  </si>
-  <si>
-    <t>PRECIO UNITARIO (PRECIO COSTO)</t>
-  </si>
-  <si>
-    <t>FACTURA Nro</t>
-  </si>
-  <si>
-    <t>Nro DE GUIA</t>
-  </si>
-  <si>
-    <t>PRECIO VTA.</t>
-  </si>
-  <si>
-    <t>PRECIO VTA. COMERCIAL</t>
-  </si>
-  <si>
-    <t>CODIGO DE BARRAS</t>
-  </si>
-  <si>
-    <t>PROVEEDOR</t>
-  </si>
-  <si>
-    <t>RUC</t>
-  </si>
-  <si>
-    <t>SEDE</t>
-  </si>
-  <si>
-    <t>F.COMPRA</t>
-  </si>
-  <si>
-    <t>REGISTRO SA.</t>
-  </si>
-  <si>
-    <t>cod_digemid</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>description</t>
-  </si>
-  <si>
-    <t>presentation</t>
-  </si>
-  <si>
-    <t>laboratorio</t>
-  </si>
-  <si>
-    <t>fecha_venc</t>
-  </si>
-  <si>
-    <t>cant_caja</t>
-  </si>
-  <si>
-    <t>stock</t>
-  </si>
-  <si>
-    <t>num_lote</t>
-  </si>
-  <si>
-    <t>prec_prov</t>
-  </si>
-  <si>
-    <t>price_in</t>
-  </si>
-  <si>
-    <t>nro_factura</t>
-  </si>
-  <si>
-    <t>nro_guia</t>
-  </si>
-  <si>
-    <t>price_out</t>
-  </si>
-  <si>
-    <t>price_may</t>
-  </si>
-  <si>
-    <t>barcode</t>
-  </si>
-  <si>
-    <t>proveedor</t>
-  </si>
-  <si>
-    <t>ruc</t>
-  </si>
-  <si>
-    <t>sede</t>
-  </si>
-  <si>
-    <t>fecha_compra</t>
-  </si>
-  <si>
-    <t>reg_san</t>
-  </si>
-  <si>
-    <t>OLCASA S.A.C.</t>
-  </si>
-  <si>
-    <t>1/25/2026</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>35167</t>
-  </si>
-  <si>
-    <t>F001-0000857</t>
-  </si>
-  <si>
-    <t>IQUITOS</t>
-  </si>
-  <si>
-    <t>5/05/2026</t>
-  </si>
-  <si>
-    <t>BICARBONATO DE SODIO</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> POTE X 50G</t>
-  </si>
-  <si>
-    <t>E-12345</t>
-  </si>
-  <si>
-    <t>ROXFARMA S.A</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
+  <si>
+    <t xml:space="preserve">COD.DIGEMID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRODUCTO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRINCIPIO ACTIVO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRESENTACION/FORMAS POR UNIDAD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LABORATORIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F.V.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CANT x CAJA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CANT. UNI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PREC.PROVEEDOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRECIO UNITARIO (PRECIO COSTO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FACTURA Nro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nro DE GUIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRECIO VTA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRECIO VTA. COMERCIAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CODIGO DE BARRAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROVEEDOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEDE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F.COMPRA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REGISTRO SA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cod_digemid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">principio_activo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">presentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">laboratorio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fecha_venc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cant_caja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stock</t>
+  </si>
+  <si>
+    <t xml:space="preserve">num_lote</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prec_prov</t>
+  </si>
+  <si>
+    <t xml:space="preserve">price_in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nro_factura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nro_guia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">price_out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">price_may</t>
+  </si>
+  <si>
+    <t xml:space="preserve">barcode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">proveedor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ruc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sede</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fecha_compra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reg_san</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1211041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BICARBONATO DE SODIO POTE X 500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BICARBONATO DE SODIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POTE X 50 GR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OLCASA S.A.C.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1/25/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35167</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S/ 15.96</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S/ 1.13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F001-0000857</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S/ 2.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S/ 1.80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.9641-15 F001-0000657</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2300657+90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IQUITOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5/05/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">123456</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="8" formatCode="&quot;S/&quot;\ #,##0.00;[Red]\-&quot;S/&quot;\ #,##0.00"/>
-  </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="4">
     <font>
       <sz val="9"/>
       <name val="Calibri"/>
@@ -198,19 +210,16 @@
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
-      <i/>
       <sz val="8"/>
       <color rgb="FF666666"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <i/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="11">
@@ -293,7 +302,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -322,536 +331,229 @@
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="8" fontId="3" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="44546A"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4472C4"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="ED7D31"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="FFC000"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="70AD47"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0563C1"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="954F72"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U103"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="8" width="14" customWidth="1"/>
-    <col min="9" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="26" customWidth="1"/>
-    <col min="13" max="13" width="18" customWidth="1"/>
-    <col min="14" max="14" width="16" customWidth="1"/>
-    <col min="15" max="15" width="14" customWidth="1"/>
-    <col min="16" max="16" width="22" customWidth="1"/>
-    <col min="17" max="17" width="20" customWidth="1"/>
-    <col min="18" max="18" width="28" customWidth="1"/>
-    <col min="19" max="19" width="16" customWidth="1"/>
-    <col min="20" max="21" width="14" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="26" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
+    <col min="15" max="15" width="22" customWidth="1"/>
+    <col min="16" max="16" width="20" customWidth="1"/>
+    <col min="17" max="17" width="28" customWidth="1"/>
+    <col min="18" max="18" width="16" customWidth="1"/>
+    <col min="19" max="19" width="14" customWidth="1"/>
+    <col min="20" max="20" width="14" customWidth="1"/>
+    <col min="21" max="21" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" t="s" s="1">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s" s="1">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s" s="1">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s" s="1">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" t="s" s="2">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" t="s" s="3">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s" s="4">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s" s="4">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s" s="4">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s" s="5">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s" s="2">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s" s="2">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s" s="6">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s" s="6">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s" s="2">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s" s="4">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s" s="3">
+        <v>19</v>
+      </c>
+      <c r="U1" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="P1" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" ht="12" x14ac:dyDescent="0.2">
-      <c r="A2" s="7" t="s">
+    </row>
+    <row r="2" ht="13">
+      <c r="A2" t="s" s="7">
         <v>21</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" t="s" s="7">
         <v>22</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" t="s" s="7">
         <v>23</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" t="s" s="7">
         <v>24</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" t="s" s="7">
         <v>25</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" t="s" s="7">
+        <v>26</v>
+      </c>
+      <c r="G2" t="s" s="7">
+        <v>27</v>
+      </c>
+      <c r="H2" t="s" s="7">
+        <v>28</v>
+      </c>
+      <c r="I2" t="s" s="7">
+        <v>29</v>
+      </c>
+      <c r="J2" t="s" s="7">
+        <v>30</v>
+      </c>
+      <c r="K2" t="s" s="7">
+        <v>31</v>
+      </c>
+      <c r="L2" t="s" s="7">
+        <v>32</v>
+      </c>
+      <c r="M2" t="s" s="7">
+        <v>33</v>
+      </c>
+      <c r="N2" t="s" s="7">
+        <v>34</v>
+      </c>
+      <c r="O2" t="s" s="7">
+        <v>35</v>
+      </c>
+      <c r="P2" t="s" s="7">
+        <v>36</v>
+      </c>
+      <c r="Q2" t="s" s="7">
+        <v>37</v>
+      </c>
+      <c r="R2" t="s" s="7">
+        <v>38</v>
+      </c>
+      <c r="S2" t="s" s="7">
+        <v>39</v>
+      </c>
+      <c r="T2" t="s" s="7">
+        <v>40</v>
+      </c>
+      <c r="U2" t="s" s="7">
         <v>41</v>
       </c>
-      <c r="G2" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="J2" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="K2" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="M2" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="N2" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="O2" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="P2" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q2" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="R2" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="S2" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="T2" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="U2" s="7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" ht="12" x14ac:dyDescent="0.2">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8" t="s">
+    </row>
+    <row r="3" ht="16">
+      <c r="A3" t="s" s="8">
+        <v>42</v>
+      </c>
+      <c r="B3" t="s" s="8">
+        <v>43</v>
+      </c>
+      <c r="C3" t="s" s="8">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s" s="8">
+        <v>45</v>
+      </c>
+      <c r="E3" t="s" s="8">
+        <v>46</v>
+      </c>
+      <c r="F3" t="s" s="8">
+        <v>47</v>
+      </c>
+      <c r="G3" t="s" s="8">
+        <v>48</v>
+      </c>
+      <c r="H3" t="s" s="8">
         <v>49</v>
       </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8" t="s">
+      <c r="I3" t="s" s="8">
         <v>50</v>
       </c>
-      <c r="E3" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="F3" s="8" t="s">
+      <c r="J3" t="s" s="8">
         <v>51</v>
       </c>
-      <c r="G3" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="H3" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="I3" s="8">
-        <v>10</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="K3" s="10">
-        <v>13.56</v>
-      </c>
-      <c r="L3" s="8">
-        <v>1.1299999999999999</v>
-      </c>
-      <c r="M3" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="N3" s="9"/>
-      <c r="O3" s="8">
-        <v>3</v>
-      </c>
-      <c r="P3" s="8">
-        <v>2.8</v>
-      </c>
-      <c r="Q3" s="8">
-        <v>77021159626955</v>
-      </c>
-      <c r="R3" s="8" t="s">
+      <c r="K3" t="s" s="8">
         <v>52</v>
       </c>
-      <c r="S3" s="9">
-        <v>20101348203</v>
-      </c>
-      <c r="T3" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="U3" s="8" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+      <c r="L3" t="s" s="8">
+        <v>53</v>
+      </c>
+      <c r="M3" s="9"/>
+      <c r="N3" t="s" s="8">
+        <v>54</v>
+      </c>
+      <c r="O3" t="s" s="8">
+        <v>55</v>
+      </c>
+      <c r="P3" t="s" s="8">
+        <v>56</v>
+      </c>
+      <c r="Q3" t="s" s="8">
+        <v>57</v>
+      </c>
+      <c r="R3" s="9"/>
+      <c r="S3" t="s" s="8">
+        <v>58</v>
+      </c>
+      <c r="T3" t="s" s="8">
+        <v>59</v>
+      </c>
+      <c r="U3" t="s" s="8">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" ht="15">
       <c r="A4" s="9"/>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
@@ -874,7 +576,7 @@
       <c r="T4" s="9"/>
       <c r="U4" s="9"/>
     </row>
-    <row r="5" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="5" ht="15">
       <c r="A5" s="9"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
@@ -897,7 +599,7 @@
       <c r="T5" s="9"/>
       <c r="U5" s="9"/>
     </row>
-    <row r="6" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="6" ht="15">
       <c r="A6" s="9"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -920,7 +622,7 @@
       <c r="T6" s="9"/>
       <c r="U6" s="9"/>
     </row>
-    <row r="7" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="7" ht="15">
       <c r="A7" s="9"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
@@ -943,7 +645,7 @@
       <c r="T7" s="9"/>
       <c r="U7" s="9"/>
     </row>
-    <row r="8" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="8" ht="15">
       <c r="A8" s="9"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -966,7 +668,7 @@
       <c r="T8" s="9"/>
       <c r="U8" s="9"/>
     </row>
-    <row r="9" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="9" ht="15">
       <c r="A9" s="9"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -989,7 +691,7 @@
       <c r="T9" s="9"/>
       <c r="U9" s="9"/>
     </row>
-    <row r="10" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="10" ht="15">
       <c r="A10" s="9"/>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -1012,7 +714,7 @@
       <c r="T10" s="9"/>
       <c r="U10" s="9"/>
     </row>
-    <row r="11" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="11" ht="15">
       <c r="A11" s="9"/>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
@@ -1035,7 +737,7 @@
       <c r="T11" s="9"/>
       <c r="U11" s="9"/>
     </row>
-    <row r="12" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="12" ht="15">
       <c r="A12" s="9"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -1058,7 +760,7 @@
       <c r="T12" s="9"/>
       <c r="U12" s="9"/>
     </row>
-    <row r="13" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="13" ht="15">
       <c r="A13" s="9"/>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -1081,7 +783,7 @@
       <c r="T13" s="9"/>
       <c r="U13" s="9"/>
     </row>
-    <row r="14" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="14" ht="15">
       <c r="A14" s="9"/>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -1104,7 +806,7 @@
       <c r="T14" s="9"/>
       <c r="U14" s="9"/>
     </row>
-    <row r="15" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="15" ht="15">
       <c r="A15" s="9"/>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -1127,7 +829,7 @@
       <c r="T15" s="9"/>
       <c r="U15" s="9"/>
     </row>
-    <row r="16" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="16" ht="15">
       <c r="A16" s="9"/>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -1150,7 +852,7 @@
       <c r="T16" s="9"/>
       <c r="U16" s="9"/>
     </row>
-    <row r="17" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="17" ht="15">
       <c r="A17" s="9"/>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
@@ -1173,7 +875,7 @@
       <c r="T17" s="9"/>
       <c r="U17" s="9"/>
     </row>
-    <row r="18" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="18" ht="15">
       <c r="A18" s="9"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -1196,7 +898,7 @@
       <c r="T18" s="9"/>
       <c r="U18" s="9"/>
     </row>
-    <row r="19" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="19" ht="15">
       <c r="A19" s="9"/>
       <c r="B19" s="9"/>
       <c r="C19" s="9"/>
@@ -1219,7 +921,7 @@
       <c r="T19" s="9"/>
       <c r="U19" s="9"/>
     </row>
-    <row r="20" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="20" ht="15">
       <c r="A20" s="9"/>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
@@ -1242,7 +944,7 @@
       <c r="T20" s="9"/>
       <c r="U20" s="9"/>
     </row>
-    <row r="21" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="21" ht="15">
       <c r="A21" s="9"/>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
@@ -1265,7 +967,7 @@
       <c r="T21" s="9"/>
       <c r="U21" s="9"/>
     </row>
-    <row r="22" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="22" ht="15">
       <c r="A22" s="9"/>
       <c r="B22" s="9"/>
       <c r="C22" s="9"/>
@@ -1288,7 +990,7 @@
       <c r="T22" s="9"/>
       <c r="U22" s="9"/>
     </row>
-    <row r="23" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="23" ht="15">
       <c r="A23" s="9"/>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
@@ -1311,7 +1013,7 @@
       <c r="T23" s="9"/>
       <c r="U23" s="9"/>
     </row>
-    <row r="24" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="24" ht="15">
       <c r="A24" s="9"/>
       <c r="B24" s="9"/>
       <c r="C24" s="9"/>
@@ -1334,7 +1036,7 @@
       <c r="T24" s="9"/>
       <c r="U24" s="9"/>
     </row>
-    <row r="25" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="25" ht="15">
       <c r="A25" s="9"/>
       <c r="B25" s="9"/>
       <c r="C25" s="9"/>
@@ -1357,7 +1059,7 @@
       <c r="T25" s="9"/>
       <c r="U25" s="9"/>
     </row>
-    <row r="26" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="26" ht="15">
       <c r="A26" s="9"/>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
@@ -1380,7 +1082,7 @@
       <c r="T26" s="9"/>
       <c r="U26" s="9"/>
     </row>
-    <row r="27" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="27" ht="15">
       <c r="A27" s="9"/>
       <c r="B27" s="9"/>
       <c r="C27" s="9"/>
@@ -1403,7 +1105,7 @@
       <c r="T27" s="9"/>
       <c r="U27" s="9"/>
     </row>
-    <row r="28" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="28" ht="15">
       <c r="A28" s="9"/>
       <c r="B28" s="9"/>
       <c r="C28" s="9"/>
@@ -1426,7 +1128,7 @@
       <c r="T28" s="9"/>
       <c r="U28" s="9"/>
     </row>
-    <row r="29" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="29" ht="15">
       <c r="A29" s="9"/>
       <c r="B29" s="9"/>
       <c r="C29" s="9"/>
@@ -1449,7 +1151,7 @@
       <c r="T29" s="9"/>
       <c r="U29" s="9"/>
     </row>
-    <row r="30" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="30" ht="15">
       <c r="A30" s="9"/>
       <c r="B30" s="9"/>
       <c r="C30" s="9"/>
@@ -1472,7 +1174,7 @@
       <c r="T30" s="9"/>
       <c r="U30" s="9"/>
     </row>
-    <row r="31" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="31" ht="15">
       <c r="A31" s="9"/>
       <c r="B31" s="9"/>
       <c r="C31" s="9"/>
@@ -1495,7 +1197,7 @@
       <c r="T31" s="9"/>
       <c r="U31" s="9"/>
     </row>
-    <row r="32" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="32" ht="15">
       <c r="A32" s="9"/>
       <c r="B32" s="9"/>
       <c r="C32" s="9"/>
@@ -1518,7 +1220,7 @@
       <c r="T32" s="9"/>
       <c r="U32" s="9"/>
     </row>
-    <row r="33" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="33" ht="15">
       <c r="A33" s="9"/>
       <c r="B33" s="9"/>
       <c r="C33" s="9"/>
@@ -1541,7 +1243,7 @@
       <c r="T33" s="9"/>
       <c r="U33" s="9"/>
     </row>
-    <row r="34" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="34" ht="15">
       <c r="A34" s="9"/>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -1564,7 +1266,7 @@
       <c r="T34" s="9"/>
       <c r="U34" s="9"/>
     </row>
-    <row r="35" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="35" ht="15">
       <c r="A35" s="9"/>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
@@ -1587,7 +1289,7 @@
       <c r="T35" s="9"/>
       <c r="U35" s="9"/>
     </row>
-    <row r="36" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="36" ht="15">
       <c r="A36" s="9"/>
       <c r="B36" s="9"/>
       <c r="C36" s="9"/>
@@ -1610,7 +1312,7 @@
       <c r="T36" s="9"/>
       <c r="U36" s="9"/>
     </row>
-    <row r="37" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="37" ht="15">
       <c r="A37" s="9"/>
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
@@ -1633,7 +1335,7 @@
       <c r="T37" s="9"/>
       <c r="U37" s="9"/>
     </row>
-    <row r="38" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="38" ht="15">
       <c r="A38" s="9"/>
       <c r="B38" s="9"/>
       <c r="C38" s="9"/>
@@ -1656,7 +1358,7 @@
       <c r="T38" s="9"/>
       <c r="U38" s="9"/>
     </row>
-    <row r="39" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="39" ht="15">
       <c r="A39" s="9"/>
       <c r="B39" s="9"/>
       <c r="C39" s="9"/>
@@ -1679,7 +1381,7 @@
       <c r="T39" s="9"/>
       <c r="U39" s="9"/>
     </row>
-    <row r="40" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="40" ht="15">
       <c r="A40" s="9"/>
       <c r="B40" s="9"/>
       <c r="C40" s="9"/>
@@ -1702,7 +1404,7 @@
       <c r="T40" s="9"/>
       <c r="U40" s="9"/>
     </row>
-    <row r="41" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="41" ht="15">
       <c r="A41" s="9"/>
       <c r="B41" s="9"/>
       <c r="C41" s="9"/>
@@ -1725,7 +1427,7 @@
       <c r="T41" s="9"/>
       <c r="U41" s="9"/>
     </row>
-    <row r="42" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="42" ht="15">
       <c r="A42" s="9"/>
       <c r="B42" s="9"/>
       <c r="C42" s="9"/>
@@ -1748,7 +1450,7 @@
       <c r="T42" s="9"/>
       <c r="U42" s="9"/>
     </row>
-    <row r="43" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="43" ht="15">
       <c r="A43" s="9"/>
       <c r="B43" s="9"/>
       <c r="C43" s="9"/>
@@ -1771,7 +1473,7 @@
       <c r="T43" s="9"/>
       <c r="U43" s="9"/>
     </row>
-    <row r="44" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="44" ht="15">
       <c r="A44" s="9"/>
       <c r="B44" s="9"/>
       <c r="C44" s="9"/>
@@ -1794,7 +1496,7 @@
       <c r="T44" s="9"/>
       <c r="U44" s="9"/>
     </row>
-    <row r="45" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="45" ht="15">
       <c r="A45" s="9"/>
       <c r="B45" s="9"/>
       <c r="C45" s="9"/>
@@ -1817,7 +1519,7 @@
       <c r="T45" s="9"/>
       <c r="U45" s="9"/>
     </row>
-    <row r="46" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="46" ht="15">
       <c r="A46" s="9"/>
       <c r="B46" s="9"/>
       <c r="C46" s="9"/>
@@ -1840,7 +1542,7 @@
       <c r="T46" s="9"/>
       <c r="U46" s="9"/>
     </row>
-    <row r="47" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="47" ht="15">
       <c r="A47" s="9"/>
       <c r="B47" s="9"/>
       <c r="C47" s="9"/>
@@ -1863,7 +1565,7 @@
       <c r="T47" s="9"/>
       <c r="U47" s="9"/>
     </row>
-    <row r="48" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="48" ht="15">
       <c r="A48" s="9"/>
       <c r="B48" s="9"/>
       <c r="C48" s="9"/>
@@ -1886,7 +1588,7 @@
       <c r="T48" s="9"/>
       <c r="U48" s="9"/>
     </row>
-    <row r="49" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="49" ht="15">
       <c r="A49" s="9"/>
       <c r="B49" s="9"/>
       <c r="C49" s="9"/>
@@ -1909,7 +1611,7 @@
       <c r="T49" s="9"/>
       <c r="U49" s="9"/>
     </row>
-    <row r="50" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="50" ht="15">
       <c r="A50" s="9"/>
       <c r="B50" s="9"/>
       <c r="C50" s="9"/>
@@ -1932,7 +1634,7 @@
       <c r="T50" s="9"/>
       <c r="U50" s="9"/>
     </row>
-    <row r="51" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="51" ht="15">
       <c r="A51" s="9"/>
       <c r="B51" s="9"/>
       <c r="C51" s="9"/>
@@ -1955,7 +1657,7 @@
       <c r="T51" s="9"/>
       <c r="U51" s="9"/>
     </row>
-    <row r="52" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="52" ht="15">
       <c r="A52" s="9"/>
       <c r="B52" s="9"/>
       <c r="C52" s="9"/>
@@ -1978,7 +1680,7 @@
       <c r="T52" s="9"/>
       <c r="U52" s="9"/>
     </row>
-    <row r="53" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="53" ht="15">
       <c r="A53" s="9"/>
       <c r="B53" s="9"/>
       <c r="C53" s="9"/>
@@ -2001,7 +1703,7 @@
       <c r="T53" s="9"/>
       <c r="U53" s="9"/>
     </row>
-    <row r="54" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="54" ht="15">
       <c r="A54" s="9"/>
       <c r="B54" s="9"/>
       <c r="C54" s="9"/>
@@ -2024,7 +1726,7 @@
       <c r="T54" s="9"/>
       <c r="U54" s="9"/>
     </row>
-    <row r="55" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="55" ht="15">
       <c r="A55" s="9"/>
       <c r="B55" s="9"/>
       <c r="C55" s="9"/>
@@ -2047,7 +1749,7 @@
       <c r="T55" s="9"/>
       <c r="U55" s="9"/>
     </row>
-    <row r="56" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="56" ht="15">
       <c r="A56" s="9"/>
       <c r="B56" s="9"/>
       <c r="C56" s="9"/>
@@ -2070,7 +1772,7 @@
       <c r="T56" s="9"/>
       <c r="U56" s="9"/>
     </row>
-    <row r="57" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="57" ht="15">
       <c r="A57" s="9"/>
       <c r="B57" s="9"/>
       <c r="C57" s="9"/>
@@ -2093,7 +1795,7 @@
       <c r="T57" s="9"/>
       <c r="U57" s="9"/>
     </row>
-    <row r="58" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="58" ht="15">
       <c r="A58" s="9"/>
       <c r="B58" s="9"/>
       <c r="C58" s="9"/>
@@ -2116,7 +1818,7 @@
       <c r="T58" s="9"/>
       <c r="U58" s="9"/>
     </row>
-    <row r="59" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="59" ht="15">
       <c r="A59" s="9"/>
       <c r="B59" s="9"/>
       <c r="C59" s="9"/>
@@ -2139,7 +1841,7 @@
       <c r="T59" s="9"/>
       <c r="U59" s="9"/>
     </row>
-    <row r="60" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="60" ht="15">
       <c r="A60" s="9"/>
       <c r="B60" s="9"/>
       <c r="C60" s="9"/>
@@ -2162,7 +1864,7 @@
       <c r="T60" s="9"/>
       <c r="U60" s="9"/>
     </row>
-    <row r="61" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="61" ht="15">
       <c r="A61" s="9"/>
       <c r="B61" s="9"/>
       <c r="C61" s="9"/>
@@ -2185,7 +1887,7 @@
       <c r="T61" s="9"/>
       <c r="U61" s="9"/>
     </row>
-    <row r="62" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="62" ht="15">
       <c r="A62" s="9"/>
       <c r="B62" s="9"/>
       <c r="C62" s="9"/>
@@ -2208,7 +1910,7 @@
       <c r="T62" s="9"/>
       <c r="U62" s="9"/>
     </row>
-    <row r="63" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="63" ht="15">
       <c r="A63" s="9"/>
       <c r="B63" s="9"/>
       <c r="C63" s="9"/>
@@ -2231,7 +1933,7 @@
       <c r="T63" s="9"/>
       <c r="U63" s="9"/>
     </row>
-    <row r="64" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="64" ht="15">
       <c r="A64" s="9"/>
       <c r="B64" s="9"/>
       <c r="C64" s="9"/>
@@ -2254,7 +1956,7 @@
       <c r="T64" s="9"/>
       <c r="U64" s="9"/>
     </row>
-    <row r="65" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="65" ht="15">
       <c r="A65" s="9"/>
       <c r="B65" s="9"/>
       <c r="C65" s="9"/>
@@ -2277,7 +1979,7 @@
       <c r="T65" s="9"/>
       <c r="U65" s="9"/>
     </row>
-    <row r="66" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="66" ht="15">
       <c r="A66" s="9"/>
       <c r="B66" s="9"/>
       <c r="C66" s="9"/>
@@ -2300,7 +2002,7 @@
       <c r="T66" s="9"/>
       <c r="U66" s="9"/>
     </row>
-    <row r="67" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="67" ht="15">
       <c r="A67" s="9"/>
       <c r="B67" s="9"/>
       <c r="C67" s="9"/>
@@ -2323,7 +2025,7 @@
       <c r="T67" s="9"/>
       <c r="U67" s="9"/>
     </row>
-    <row r="68" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="68" ht="15">
       <c r="A68" s="9"/>
       <c r="B68" s="9"/>
       <c r="C68" s="9"/>
@@ -2346,7 +2048,7 @@
       <c r="T68" s="9"/>
       <c r="U68" s="9"/>
     </row>
-    <row r="69" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="69" ht="15">
       <c r="A69" s="9"/>
       <c r="B69" s="9"/>
       <c r="C69" s="9"/>
@@ -2369,7 +2071,7 @@
       <c r="T69" s="9"/>
       <c r="U69" s="9"/>
     </row>
-    <row r="70" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="70" ht="15">
       <c r="A70" s="9"/>
       <c r="B70" s="9"/>
       <c r="C70" s="9"/>
@@ -2392,7 +2094,7 @@
       <c r="T70" s="9"/>
       <c r="U70" s="9"/>
     </row>
-    <row r="71" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="71" ht="15">
       <c r="A71" s="9"/>
       <c r="B71" s="9"/>
       <c r="C71" s="9"/>
@@ -2415,7 +2117,7 @@
       <c r="T71" s="9"/>
       <c r="U71" s="9"/>
     </row>
-    <row r="72" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="72" ht="15">
       <c r="A72" s="9"/>
       <c r="B72" s="9"/>
       <c r="C72" s="9"/>
@@ -2438,7 +2140,7 @@
       <c r="T72" s="9"/>
       <c r="U72" s="9"/>
     </row>
-    <row r="73" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="73" ht="15">
       <c r="A73" s="9"/>
       <c r="B73" s="9"/>
       <c r="C73" s="9"/>
@@ -2461,7 +2163,7 @@
       <c r="T73" s="9"/>
       <c r="U73" s="9"/>
     </row>
-    <row r="74" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="74" ht="15">
       <c r="A74" s="9"/>
       <c r="B74" s="9"/>
       <c r="C74" s="9"/>
@@ -2484,7 +2186,7 @@
       <c r="T74" s="9"/>
       <c r="U74" s="9"/>
     </row>
-    <row r="75" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="75" ht="15">
       <c r="A75" s="9"/>
       <c r="B75" s="9"/>
       <c r="C75" s="9"/>
@@ -2507,7 +2209,7 @@
       <c r="T75" s="9"/>
       <c r="U75" s="9"/>
     </row>
-    <row r="76" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="76" ht="15">
       <c r="A76" s="9"/>
       <c r="B76" s="9"/>
       <c r="C76" s="9"/>
@@ -2530,7 +2232,7 @@
       <c r="T76" s="9"/>
       <c r="U76" s="9"/>
     </row>
-    <row r="77" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="77" ht="15">
       <c r="A77" s="9"/>
       <c r="B77" s="9"/>
       <c r="C77" s="9"/>
@@ -2553,7 +2255,7 @@
       <c r="T77" s="9"/>
       <c r="U77" s="9"/>
     </row>
-    <row r="78" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="78" ht="15">
       <c r="A78" s="9"/>
       <c r="B78" s="9"/>
       <c r="C78" s="9"/>
@@ -2576,7 +2278,7 @@
       <c r="T78" s="9"/>
       <c r="U78" s="9"/>
     </row>
-    <row r="79" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="79" ht="15">
       <c r="A79" s="9"/>
       <c r="B79" s="9"/>
       <c r="C79" s="9"/>
@@ -2599,7 +2301,7 @@
       <c r="T79" s="9"/>
       <c r="U79" s="9"/>
     </row>
-    <row r="80" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="80" ht="15">
       <c r="A80" s="9"/>
       <c r="B80" s="9"/>
       <c r="C80" s="9"/>
@@ -2622,7 +2324,7 @@
       <c r="T80" s="9"/>
       <c r="U80" s="9"/>
     </row>
-    <row r="81" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="81" ht="15">
       <c r="A81" s="9"/>
       <c r="B81" s="9"/>
       <c r="C81" s="9"/>
@@ -2645,7 +2347,7 @@
       <c r="T81" s="9"/>
       <c r="U81" s="9"/>
     </row>
-    <row r="82" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="82" ht="15">
       <c r="A82" s="9"/>
       <c r="B82" s="9"/>
       <c r="C82" s="9"/>
@@ -2668,7 +2370,7 @@
       <c r="T82" s="9"/>
       <c r="U82" s="9"/>
     </row>
-    <row r="83" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="83" ht="15">
       <c r="A83" s="9"/>
       <c r="B83" s="9"/>
       <c r="C83" s="9"/>
@@ -2691,7 +2393,7 @@
       <c r="T83" s="9"/>
       <c r="U83" s="9"/>
     </row>
-    <row r="84" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="84" ht="15">
       <c r="A84" s="9"/>
       <c r="B84" s="9"/>
       <c r="C84" s="9"/>
@@ -2714,7 +2416,7 @@
       <c r="T84" s="9"/>
       <c r="U84" s="9"/>
     </row>
-    <row r="85" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="85" ht="15">
       <c r="A85" s="9"/>
       <c r="B85" s="9"/>
       <c r="C85" s="9"/>
@@ -2737,7 +2439,7 @@
       <c r="T85" s="9"/>
       <c r="U85" s="9"/>
     </row>
-    <row r="86" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="86" ht="15">
       <c r="A86" s="9"/>
       <c r="B86" s="9"/>
       <c r="C86" s="9"/>
@@ -2760,7 +2462,7 @@
       <c r="T86" s="9"/>
       <c r="U86" s="9"/>
     </row>
-    <row r="87" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="87" ht="15">
       <c r="A87" s="9"/>
       <c r="B87" s="9"/>
       <c r="C87" s="9"/>
@@ -2783,7 +2485,7 @@
       <c r="T87" s="9"/>
       <c r="U87" s="9"/>
     </row>
-    <row r="88" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="88" ht="15">
       <c r="A88" s="9"/>
       <c r="B88" s="9"/>
       <c r="C88" s="9"/>
@@ -2806,7 +2508,7 @@
       <c r="T88" s="9"/>
       <c r="U88" s="9"/>
     </row>
-    <row r="89" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="89" ht="15">
       <c r="A89" s="9"/>
       <c r="B89" s="9"/>
       <c r="C89" s="9"/>
@@ -2829,7 +2531,7 @@
       <c r="T89" s="9"/>
       <c r="U89" s="9"/>
     </row>
-    <row r="90" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="90" ht="15">
       <c r="A90" s="9"/>
       <c r="B90" s="9"/>
       <c r="C90" s="9"/>
@@ -2852,7 +2554,7 @@
       <c r="T90" s="9"/>
       <c r="U90" s="9"/>
     </row>
-    <row r="91" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="91" ht="15">
       <c r="A91" s="9"/>
       <c r="B91" s="9"/>
       <c r="C91" s="9"/>
@@ -2875,7 +2577,7 @@
       <c r="T91" s="9"/>
       <c r="U91" s="9"/>
     </row>
-    <row r="92" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="92" ht="15">
       <c r="A92" s="9"/>
       <c r="B92" s="9"/>
       <c r="C92" s="9"/>
@@ -2898,7 +2600,7 @@
       <c r="T92" s="9"/>
       <c r="U92" s="9"/>
     </row>
-    <row r="93" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="93" ht="15">
       <c r="A93" s="9"/>
       <c r="B93" s="9"/>
       <c r="C93" s="9"/>
@@ -2921,7 +2623,7 @@
       <c r="T93" s="9"/>
       <c r="U93" s="9"/>
     </row>
-    <row r="94" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="94" ht="15">
       <c r="A94" s="9"/>
       <c r="B94" s="9"/>
       <c r="C94" s="9"/>
@@ -2944,7 +2646,7 @@
       <c r="T94" s="9"/>
       <c r="U94" s="9"/>
     </row>
-    <row r="95" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="95" ht="15">
       <c r="A95" s="9"/>
       <c r="B95" s="9"/>
       <c r="C95" s="9"/>
@@ -2967,7 +2669,7 @@
       <c r="T95" s="9"/>
       <c r="U95" s="9"/>
     </row>
-    <row r="96" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="96" ht="15">
       <c r="A96" s="9"/>
       <c r="B96" s="9"/>
       <c r="C96" s="9"/>
@@ -2990,7 +2692,7 @@
       <c r="T96" s="9"/>
       <c r="U96" s="9"/>
     </row>
-    <row r="97" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="97" ht="15">
       <c r="A97" s="9"/>
       <c r="B97" s="9"/>
       <c r="C97" s="9"/>
@@ -3013,7 +2715,7 @@
       <c r="T97" s="9"/>
       <c r="U97" s="9"/>
     </row>
-    <row r="98" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="98" ht="15">
       <c r="A98" s="9"/>
       <c r="B98" s="9"/>
       <c r="C98" s="9"/>
@@ -3036,7 +2738,7 @@
       <c r="T98" s="9"/>
       <c r="U98" s="9"/>
     </row>
-    <row r="99" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="99" ht="15">
       <c r="A99" s="9"/>
       <c r="B99" s="9"/>
       <c r="C99" s="9"/>
@@ -3059,7 +2761,7 @@
       <c r="T99" s="9"/>
       <c r="U99" s="9"/>
     </row>
-    <row r="100" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="100" ht="15">
       <c r="A100" s="9"/>
       <c r="B100" s="9"/>
       <c r="C100" s="9"/>
@@ -3082,7 +2784,7 @@
       <c r="T100" s="9"/>
       <c r="U100" s="9"/>
     </row>
-    <row r="101" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="101" ht="15">
       <c r="A101" s="9"/>
       <c r="B101" s="9"/>
       <c r="C101" s="9"/>
@@ -3105,7 +2807,7 @@
       <c r="T101" s="9"/>
       <c r="U101" s="9"/>
     </row>
-    <row r="102" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="102" ht="15">
       <c r="A102" s="9"/>
       <c r="B102" s="9"/>
       <c r="C102" s="9"/>
@@ -3128,7 +2830,7 @@
       <c r="T102" s="9"/>
       <c r="U102" s="9"/>
     </row>
-    <row r="103" spans="1:21" ht="12" x14ac:dyDescent="0.2">
+    <row r="103" ht="15">
       <c r="A103" s="9"/>
       <c r="B103" s="9"/>
       <c r="C103" s="9"/>
@@ -3152,7 +2854,6 @@
       <c r="U103" s="9"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
+  <pageSetup orientation="landscape" paperSize="9"/>
 </worksheet>
 </file>
</xml_diff>